<commit_message>
Dejo lo basico, me voy a dormir, preparo bien la teoria y listo
</commit_message>
<xml_diff>
--- a/Pruebas.xlsx
+++ b/Pruebas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tensi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Documents\GitHub\sew-25-26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6667ECCC-B03F-43AE-BED4-EDFD32D0271B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD64EA0-C5F2-4834-8912-9443A3DF6589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5250" yWindow="0" windowWidth="15750" windowHeight="11055" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
   <si>
     <t>Prueba</t>
   </si>
@@ -84,18 +84,12 @@
     <t>Resultado</t>
   </si>
   <si>
-    <t>Dime cuantos enlances a redes tiene</t>
-  </si>
-  <si>
     <t>Quien es el desarrollador de la web</t>
   </si>
   <si>
     <t>Completa el tiempo del juego de memoria e indica el tiempo que tardaste</t>
   </si>
   <si>
-    <t>Pon en marcha un juego de cronometraje, paralo y reinicialo.</t>
-  </si>
-  <si>
     <t>Indica cuando es la puesta del sol el día de la carrera</t>
   </si>
   <si>
@@ -138,29 +132,62 @@
     <t>Franco Morbidelli</t>
   </si>
   <si>
-    <t>3 enlaces</t>
-  </si>
-  <si>
-    <t>Diego Martínez</t>
-  </si>
-  <si>
-    <t>00:28.2</t>
-  </si>
-  <si>
-    <t>Ok</t>
-  </si>
-  <si>
     <t>Las coordenadas se podrían incluir en el apartado de circuito, y tampoco podía encontrar ña segunda escudería</t>
   </si>
   <si>
     <t>Resaltar la parte de segunda escudería</t>
+  </si>
+  <si>
+    <t>Dime cuantos enlances a redes sociales tiene el piloto</t>
+  </si>
+  <si>
+    <t>Pon en marcha un juego de cronometraje, paralo y reinicialo, avisa para hacerlo</t>
+  </si>
+  <si>
+    <t>SemiJubilada</t>
+  </si>
+  <si>
+    <t>Ordenador</t>
+  </si>
+  <si>
+    <t>Abandona</t>
+  </si>
+  <si>
+    <t>No sabe lo que es la escudería</t>
+  </si>
+  <si>
+    <t>Fácil de entender, alguna cosa poco intuitiva como las coordenadas o loas archivos que hay que adjuntar en el apartado "circuitos"</t>
+  </si>
+  <si>
+    <t>Colocar las cordenadas y la ubicación del circuito en el apartado "circuito" y no en meteorología.</t>
+  </si>
+  <si>
+    <t>Acierto</t>
+  </si>
+  <si>
+    <t>Teleoperador</t>
+  </si>
+  <si>
+    <t>Diego Martínez Menéndez</t>
+  </si>
+  <si>
+    <t>Petarmina</t>
+  </si>
+  <si>
+    <t>16.608333333333, 49.195277777778</t>
+  </si>
+  <si>
+    <t>Díficil de encontrar segunda escuderia.</t>
+  </si>
+  <si>
+    <t>Explicar un poco mejor algunas preguntas</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,6 +202,18 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -197,14 +236,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,15 +652,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.875" customWidth="1"/>
-    <col min="3" max="3" width="15.875" customWidth="1"/>
-    <col min="5" max="5" width="15.625" customWidth="1"/>
-    <col min="6" max="6" width="32.375" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -632,7 +680,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -640,220 +688,256 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D2">
         <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D3">
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D4">
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D5">
         <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F5">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6">
+        <v>47</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -869,189 +953,189 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.375" customWidth="1"/>
-    <col min="2" max="2" width="81" style="4" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="81" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.5">
+    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1066,19 +1150,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.125" customWidth="1"/>
-    <col min="2" max="2" width="14.75" customWidth="1"/>
-    <col min="3" max="3" width="24.125" customWidth="1"/>
-    <col min="4" max="4" width="25.75" customWidth="1"/>
-    <col min="5" max="5" width="26.125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="26.875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="48" style="3" customWidth="1"/>
+    <col min="6" max="6" width="40.28515625" style="3" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1091,45 +1175,45 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="57">
+    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C2">
         <v>7.46</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>30</v>
+      <c r="E2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="G2">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="42.75">
+    <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C3">
         <v>18.260000000000002</v>
@@ -1137,33 +1221,33 @@
       <c r="D3">
         <v>90</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>33</v>
+      <c r="E3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="G3">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C4">
         <v>13.44</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="71.25">
+    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>10.130000000000001</v>
@@ -1171,14 +1255,77 @@
       <c r="D5">
         <v>90</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>41</v>
+      <c r="E5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="G5">
         <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6">
+        <v>26.41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7">
+        <v>11.44</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8">
+        <v>7.57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1192,13 +1339,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="64.125" customWidth="1"/>
+    <col min="2" max="2" width="72" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1209,114 +1356,116 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="C2" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="C3" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>18</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>19</v>
+      </c>
+      <c r="C5" s="5">
+        <v>3.4953703703703704E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>37</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="2">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5">
         <v>0.75763888888888886</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+        <v>22</v>
+      </c>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="7">
         <v>0.27</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2">
+        <v>23</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="4"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ediciones para tanda 2 y validación pasada
</commit_message>
<xml_diff>
--- a/Pruebas.xlsx
+++ b/Pruebas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Documents\GitHub\sew-25-26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7FAC14-3AD0-4977-AA63-7F60B9B2FD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1AE0F3-8D51-48F7-AE86-5F05235AFE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
   <si>
     <t>ID</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Tanda</t>
   </si>
   <si>
-    <t>Estudiante</t>
-  </si>
-  <si>
     <t>Masculino</t>
   </si>
   <si>
@@ -126,6 +123,36 @@
   </si>
   <si>
     <t xml:space="preserve"> (Abandono) 1:57</t>
+  </si>
+  <si>
+    <t>Estudiante - Construcciones Metalicas</t>
+  </si>
+  <si>
+    <t>Estudiante - Instalaciones Electricas</t>
+  </si>
+  <si>
+    <t>Estudiante - Enfermeria</t>
+  </si>
+  <si>
+    <t>Estudiante - Ing. Infor</t>
+  </si>
+  <si>
+    <t>Pagina intuitiva, util y facil de buscar la información.</t>
+  </si>
+  <si>
+    <t>No ve cambios de mejora</t>
+  </si>
+  <si>
+    <t>El color de la pagina no le convence del todo.</t>
+  </si>
+  <si>
+    <t>Que el texto no sea tan plano, se nota mucho en las rutas.</t>
+  </si>
+  <si>
+    <t>Este usuario tiene TDAH, viendo que tuvo problemas para encontrar en la primera tarea la respuesta de la pregunta 4 de sacar el productor de la tabla. Al finalizar la prueba con todo aciertos menos en esa, se le indica que revise bien la página, se lo toma con algo más de calma, y saca la respues, aunque esto no se tuvo en cuenta para las mediciones o resultados. En la tarea 2, pasa varias veces por el mismo sitio, hasta que se da cuenta de que era eso, y se llama insulta por no fijarse, pues se veía facilmente bajo su punto de vista. En la ultima actividad, el usuario fue directo a iniciar sesión, le dió fallo y entonces va a registrarse. Cuando termina de registrarse, consulta recursos, y realiza la reserva despues de consultar el presupuesto.</t>
+  </si>
+  <si>
+    <t>Este usuario no ha tenido problemas para nada, todo lo ha resuelto con rapidez, se atascó solamente en la primera pregunta del juego y luego a la hora de hacer las reservas, donde va directamente a ver los recursos, se le indica iniciar sesión, y cuando le sale la vista de registro, se asusta, vuelve atrás, y vuelve a entrar. Ve que está bien, realiza el registro y finaliza la reserva normal, solicitando primero el presupuesto.</t>
   </si>
 </sst>
 </file>
@@ -133,7 +160,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="h:mm;@"/>
+    <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -182,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -194,19 +221,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -215,7 +245,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -251,7 +281,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:I1048576" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID Usuario"/>
@@ -273,7 +303,7 @@
   <autoFilter ref="A1:B1048576" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID Usuario"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -600,7 +630,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" customWidth="1"/>
     <col min="6" max="6" width="32.42578125" customWidth="1"/>
   </cols>
@@ -633,13 +663,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D2">
         <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -653,13 +683,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D3">
         <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3">
         <v>8</v>
@@ -673,13 +703,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4">
         <v>4</v>
@@ -693,13 +723,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5">
         <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -712,6 +742,18 @@
       <c r="B6">
         <v>2</v>
       </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -719,6 +761,18 @@
       </c>
       <c r="B7">
         <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -799,16 +853,16 @@
         <v>7</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>8</v>
@@ -825,7 +879,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" s="5">
         <v>9.375E-2</v>
@@ -833,17 +887,17 @@
       <c r="D2">
         <v>10</v>
       </c>
-      <c r="E2" s="7">
-        <v>14</v>
+      <c r="E2" s="9">
+        <v>9.7222222222222224E-3</v>
       </c>
       <c r="F2" s="6">
         <v>3.9583333333333331E-2</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -851,7 +905,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="5">
         <v>0.13541666666666666</v>
@@ -859,17 +913,17 @@
       <c r="D3">
         <v>9</v>
       </c>
-      <c r="E3" s="7">
-        <v>33</v>
+      <c r="E3" s="9">
+        <v>2.2916666666666665E-2</v>
       </c>
       <c r="F3" s="6">
         <v>0.30972222222222223</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -877,7 +931,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="5">
         <v>0.33333333333333331</v>
@@ -885,17 +939,17 @@
       <c r="D4">
         <v>7</v>
       </c>
-      <c r="E4" s="7">
-        <v>43</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>32</v>
+      <c r="E4" s="9">
+        <v>2.9861111111111113E-2</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -903,37 +957,69 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0.12083333333333333</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="F6" s="5">
+        <v>5.4166666666666669E-2</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="5"/>
+        <v>14</v>
+      </c>
+      <c r="C7" s="10">
+        <v>0.15277777777777779</v>
+      </c>
+      <c r="D7">
+        <v>9</v>
+      </c>
+      <c r="E7" s="8">
+        <v>6.3888888888888884E-2</v>
+      </c>
+      <c r="F7" s="5">
+        <v>3.888888888888889E-2</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="5"/>
@@ -943,7 +1029,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="5"/>
@@ -953,7 +1039,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="5"/>
@@ -963,7 +1049,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="5"/>
@@ -973,7 +1059,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="5"/>
@@ -983,7 +1069,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="5"/>
@@ -999,14 +1085,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
     <col min="2" max="2" width="81" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1014,86 +1100,93 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="150" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Listo para tanda 3
</commit_message>
<xml_diff>
--- a/Pruebas.xlsx
+++ b/Pruebas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Documents\GitHub\sew-25-26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1AE0F3-8D51-48F7-AE86-5F05235AFE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EFBCD0-D755-4F5B-8867-54AB9F8ABD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="51">
   <si>
     <t>ID</t>
   </si>
@@ -153,6 +153,33 @@
   </si>
   <si>
     <t>Este usuario no ha tenido problemas para nada, todo lo ha resuelto con rapidez, se atascó solamente en la primera pregunta del juego y luego a la hora de hacer las reservas, donde va directamente a ver los recursos, se le indica iniciar sesión, y cuando le sale la vista de registro, se asusta, vuelve atrás, y vuelve a entrar. Ve que está bien, realiza el registro y finaliza la reserva normal, solicitando primero el presupuesto.</t>
+  </si>
+  <si>
+    <t>Carpintero</t>
+  </si>
+  <si>
+    <t>Maculino</t>
+  </si>
+  <si>
+    <t>Se ve bien y se maneja sin problemas, lo unico que costó fue reservar una activcidad, que no me dejaba porque nio había plazas y no se notificaba bien.</t>
+  </si>
+  <si>
+    <t>Mejorar la notificación de plazas agotadas o limitarla. Intentar cambiar un poco los colores, hay pocos y en rutas se vería mejor con más colores. Si una ruta tiene 0 plazas sigue apareciendo, evitar eso.</t>
+  </si>
+  <si>
+    <t>Paro - Grado Sup. Infor</t>
+  </si>
+  <si>
+    <t>Lo unico que me costó saber fue que era un desplegable en la rutas</t>
+  </si>
+  <si>
+    <t>Nada a mejorar</t>
+  </si>
+  <si>
+    <t>No es una pagina muy intuitiva. No sabes muy bien cuando has realizado una acción y cuando no. La búsqueda de información de las rutas es tedioso.</t>
+  </si>
+  <si>
+    <t>Como mejora para las rutas, dejarlas por separado por enlaces. Que el registro te inicie la sesión.</t>
   </si>
 </sst>
 </file>
@@ -209,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -226,10 +253,8 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -242,10 +267,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -281,7 +306,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:I1048576" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID Usuario"/>
@@ -290,8 +315,8 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Ejercicio 1 - Puntuación  "/>
     <tableColumn id="11" xr3:uid="{8B85C65B-D1B3-46AE-A24F-230E04FA8B0C}" name="Ejercici 2 - Tiempo"/>
     <tableColumn id="8" xr3:uid="{90F54C5C-90B9-4ACC-8AE6-D36E0D6960D3}" name="Ejercicio 3 - Tiempo"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Comentarios del usuario" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Propuesta de mejora" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Comentarios del usuario" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Propuesta de mejora" dataDxfId="0"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Valoración del usuario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -303,7 +328,7 @@
   <autoFilter ref="A1:B1048576" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID Usuario"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -692,7 +717,7 @@
         <v>13</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -782,6 +807,18 @@
       <c r="B8">
         <v>2</v>
       </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -789,6 +826,18 @@
       </c>
       <c r="B9">
         <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -887,7 +936,7 @@
       <c r="D2">
         <v>10</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>9.7222222222222224E-3</v>
       </c>
       <c r="F2" s="6">
@@ -913,7 +962,7 @@
       <c r="D3">
         <v>9</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>2.2916666666666665E-2</v>
       </c>
       <c r="F3" s="6">
@@ -939,7 +988,7 @@
       <c r="D4">
         <v>7</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>2.9861111111111113E-2</v>
       </c>
       <c r="F4" s="7" t="s">
@@ -952,15 +1001,31 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="5"/>
+      <c r="C5" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1.9444444444444445E-2</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0.11319444444444444</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -969,7 +1034,7 @@
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>0.12083333333333333</v>
       </c>
       <c r="D6">
@@ -978,7 +1043,7 @@
       <c r="E6" s="8">
         <v>1.3888888888888888E-2</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="6">
         <v>5.4166666666666669E-2</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -995,7 +1060,7 @@
       <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>0.15277777777777779</v>
       </c>
       <c r="D7">
@@ -1004,7 +1069,7 @@
       <c r="E7" s="8">
         <v>6.3888888888888884E-2</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="6">
         <v>3.888888888888889E-2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -1014,25 +1079,57 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8" s="9">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8" s="8">
+        <v>4.8611111111111112E-3</v>
+      </c>
+      <c r="F8" s="6">
+        <v>5.347222222222222E-2</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="5"/>
+      <c r="C9" s="9">
+        <v>0.19791666666666666</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="F9" s="6">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1085,14 +1182,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
     <col min="2" max="2" width="81" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1100,7 +1197,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1108,7 +1205,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1116,7 +1213,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="150" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1124,21 +1221,20 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="11"/>
-    </row>
-    <row r="7" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1146,47 +1242,47 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Finalización de la tanda 3
</commit_message>
<xml_diff>
--- a/Pruebas.xlsx
+++ b/Pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Documents\GitHub\sew-25-26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EFBCD0-D755-4F5B-8867-54AB9F8ABD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F548F8-E277-4D9E-AC44-A46485DA9BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Se ve bien y se maneja sin problemas, lo unico que costó fue reservar una activcidad, que no me dejaba porque nio había plazas y no se notificaba bien.</t>
   </si>
   <si>
-    <t>Mejorar la notificación de plazas agotadas o limitarla. Intentar cambiar un poco los colores, hay pocos y en rutas se vería mejor con más colores. Si una ruta tiene 0 plazas sigue apareciendo, evitar eso.</t>
-  </si>
-  <si>
     <t>Paro - Grado Sup. Infor</t>
   </si>
   <si>
@@ -180,6 +177,60 @@
   </si>
   <si>
     <t>Como mejora para las rutas, dejarlas por separado por enlaces. Que el registro te inicie la sesión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camarera </t>
+  </si>
+  <si>
+    <t>Está conforme con la web, es facil e intuitiva, y se ven bien las cosas.</t>
+  </si>
+  <si>
+    <t>Este usuario ya hizo más test para la evaluación continua, el comentario de este usuario ha sido que le ha resultado más facil encotnrar toda la información y navegar por la web. En la primera vez que se le llamó, era la primera tanda del proyecto, por lo que es normal que este usuario note que esta web está mejor programada que la anterior, y que tiene un mayor sentido lógico. En la primer tarea no se obserbó ninguna anomalia, el usuario poco a poco saco todo sin problema, si que es verdad que en la actividad 2, el usuario se atascó a la hora de encontrar la ruta que se le indicaba en la tarea, pero una vez que se dió cuenta, dijo que no se había fijado pero que estaba facil de ver. En la ultima tarea, procedimientos limpios sin errores.</t>
+  </si>
+  <si>
+    <t>Este usurio respondió sin problemas a las cuestiones de la primera y segunda actividad. En la ultima en cambio, tuvo problemas porque no se daba cuenta de que no podía reservar 3 plazas cuando el maximo disponible era de 2, por lo que no veía la alerta y se queda atascado.</t>
+  </si>
+  <si>
+    <t>Este usuario, al estar en opera, el navegador le dificultó identificar que las rutas se cogían a partir de un desplegable, pero una vez que detectó eso, poco a poco fue sacando las cosas. Se observa que es una persona tambien con TDHA, los resultados se obtienen de apoco, pero sin mucho problema en cuanto a buscar la información.</t>
+  </si>
+  <si>
+    <t>Estudiante - Ing. Computación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejorar la notificación de plazas agotadas o limitarla. Intentar cambiar un poco los colores, hay pocos y en rutas se vería mejor con más colores. </t>
+  </si>
+  <si>
+    <t>Si una ruta tiene 0 plazas sigue apareciendo, evitar eso. Colores más bonitos de diseño.</t>
+  </si>
+  <si>
+    <t>Facil y practica, pagina intuitiva, solamente que hay momentos en los que la pagina tiene el contenido muy pequeño. Lo colores no combinan. Está muy bien el tener la opcion de registrarse cuando estás dentro de los recursos para reservar, evitas pulsaciones innecesarias.</t>
+  </si>
+  <si>
+    <t>Militar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es intuitiva y esta bien organizada, pero tiene un estilo visual algo simple y anticuado, propio de paginas web antiguas. </t>
+  </si>
+  <si>
+    <t>Mejorar el diseño y poner las rutas en un desplegable del nav de rutas.</t>
+  </si>
+  <si>
+    <t>Estudiante - Anatomia y Laboratorio</t>
+  </si>
+  <si>
+    <t>Se encuentra facil toda la información, está a la vista.</t>
+  </si>
+  <si>
+    <t>El usuario se desenvuelve bien con las actividades, procesos rápidos, claros. La unica observación es que se dio cuenta de un fallo en el que se puede intentar reservar una actividad con 0 plazas reservables.</t>
+  </si>
+  <si>
+    <t>El usuario realiza las tareas con calma, lee en voz alta lo que pasa por su cabeza. La primera tarea la realiza con calma paso a paso, pero en la parte de los hitos y de las rutas se lia, no sabe lo que es un hito realmente, aunque al final se da cuenta y  responde. El fallo que tiene en el cuestionario es porque no sabía comparar la altura de los hitos de la ruta. En la ultima prueba, el usuario tarda porque quiere mirar las actividades que hay y quiere saber cual le gustaría mas, pero se maneja con agilidad por el sitio web.</t>
+  </si>
+  <si>
+    <t>Esta persona está nervisosa al principio, le cuesta arrancar a hacer las tareas del ejercicio 1, pero cuando coge confianza, realiza las tareas con velocidad, se acostumbra a la página. Por lo demás, no hay novedades, al igual que el usuario 11, se para a mirar las actividades que hay para reservar la actividad que más le gusta.</t>
+  </si>
+  <si>
+    <t>El diseño podría mejorase, hacerlo más elegante y usar más colores pastel.</t>
   </si>
 </sst>
 </file>
@@ -189,7 +240,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,25 +254,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFD6763"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -241,7 +287,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -249,12 +294,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="20" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -267,10 +313,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -306,7 +352,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:I1048576" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="ID Usuario"/>
@@ -315,8 +361,8 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Ejercicio 1 - Puntuación  "/>
     <tableColumn id="11" xr3:uid="{8B85C65B-D1B3-46AE-A24F-230E04FA8B0C}" name="Ejercici 2 - Tiempo"/>
     <tableColumn id="8" xr3:uid="{90F54C5C-90B9-4ACC-8AE6-D36E0D6960D3}" name="Ejercicio 3 - Tiempo"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Comentarios del usuario" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Propuesta de mejora" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Comentarios del usuario" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Propuesta de mejora" dataDxfId="1"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Valoración del usuario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -328,7 +374,7 @@
   <autoFilter ref="A1:B1048576" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID Usuario"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Comentario" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -737,7 +783,7 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -808,7 +854,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8">
         <v>28</v>
@@ -847,6 +893,18 @@
       <c r="B10">
         <v>3</v>
       </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -855,6 +913,18 @@
       <c r="B11">
         <v>3</v>
       </c>
+      <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -863,6 +933,18 @@
       <c r="B12">
         <v>3</v>
       </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12">
+        <v>6</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -870,6 +952,18 @@
       </c>
       <c r="B13">
         <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -895,31 +989,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -930,16 +1024,16 @@
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>9.375E-2</v>
       </c>
       <c r="D2">
         <v>10</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="7">
         <v>9.7222222222222224E-3</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="8">
         <v>3.9583333333333331E-2</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -947,6 +1041,9 @@
       </c>
       <c r="H2" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="I2">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -956,16 +1053,16 @@
       <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <v>0.13541666666666666</v>
       </c>
       <c r="D3">
         <v>9</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <v>2.2916666666666665E-2</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="8">
         <v>0.30972222222222223</v>
       </c>
       <c r="G3" s="1" t="s">
@@ -973,6 +1070,9 @@
       </c>
       <c r="H3" s="1" t="s">
         <v>20</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -982,16 +1082,16 @@
       <c r="B4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>0.33333333333333331</v>
       </c>
       <c r="D4">
         <v>7</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <v>2.9861111111111113E-2</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="9" t="s">
         <v>31</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -999,6 +1099,9 @@
       </c>
       <c r="H4" s="1" t="s">
         <v>24</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -1008,23 +1111,26 @@
       <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="5">
         <v>0.15</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <v>1.9444444444444445E-2</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="8">
         <v>0.11319444444444444</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>50</v>
+      <c r="I5">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1034,16 +1140,16 @@
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="5">
         <v>0.12083333333333333</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>1.3888888888888888E-2</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="8">
         <v>5.4166666666666669E-2</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -1051,6 +1157,9 @@
       </c>
       <c r="H6" s="1" t="s">
         <v>37</v>
+      </c>
+      <c r="I6">
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1060,16 +1169,16 @@
       <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="5">
         <v>0.15277777777777779</v>
       </c>
       <c r="D7">
         <v>9</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <v>6.3888888888888884E-2</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="8">
         <v>3.888888888888889E-2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -1078,31 +1187,37 @@
       <c r="H7" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="5">
         <v>6.9444444444444448E-2</v>
       </c>
       <c r="D8">
         <v>10</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>4.8611111111111112E-3</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="8">
         <v>5.347222222222222E-2</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>44</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>45</v>
+        <v>56</v>
+      </c>
+      <c r="I8">
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1112,64 +1227,143 @@
       <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="5">
         <v>0.19791666666666666</v>
       </c>
       <c r="D9">
         <v>10</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <v>0.05</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="8">
         <v>7.5694444444444439E-2</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C10" s="5">
+        <v>0.15277777777777779</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10" s="7">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="F10" s="8">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="5">
+        <v>0.11388888888888889</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11" s="7">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="F11" s="8">
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C12" s="5">
+        <v>0.23541666666666666</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12" s="7">
+        <v>2.7083333333333334E-2</v>
+      </c>
+      <c r="F12" s="8">
+        <v>8.8888888888888892E-2</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="5"/>
+      <c r="C13" s="5">
+        <v>0.21319444444444444</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1.1111111111111112E-2</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0.10902777777777778</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1242,34 +1436,52 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>